<commit_message>
premier jet automne 2026
</commit_message>
<xml_diff>
--- a/template/equipe.xlsx
+++ b/template/equipe.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/etiennerivard/notes_de_cours/techinfo/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B77657A-0850-3F4C-A0F6-735295A31A32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F528629-C33B-AC4C-8E35-71F2265057B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17620" xr2:uid="{6B795B45-6C14-B04F-B93D-A59A5BE3A68D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="38">
   <si>
     <t>nom</t>
   </si>
@@ -98,15 +98,6 @@
     <t>https://teams.microsoft.com/l/chat/0/0?tenantId=9d6cf526-ad81-46f8-a73a-a507aaf06cda&amp;users=FRECHETTE.MATHIEU@cegepvicto.ca</t>
   </si>
   <si>
-    <t>Christiane Lagacé</t>
-  </si>
-  <si>
-    <t>lagace.christiane@cegepvicto.ca</t>
-  </si>
-  <si>
-    <t>https://teams.microsoft.com/l/chat/0/0?tenantId=9d6cf526-ad81-46f8-a73a-a507aaf06cda&amp;users=LAGACE.CHRISTIANE@cegepvicto.ca</t>
-  </si>
-  <si>
     <t>François Mercier</t>
   </si>
   <si>
@@ -143,9 +134,6 @@
     <t>/assets/mathieu-frechette.jpeg</t>
   </si>
   <si>
-    <t>/assets/christiane-lagace.jpeg</t>
-  </si>
-  <si>
     <t>/assets/frederik-taleb.jpeg</t>
   </si>
   <si>
@@ -153,6 +141,15 @@
   </si>
   <si>
     <t>/assets/francois-mercier.png</t>
+  </si>
+  <si>
+    <t>Sébastien Trottier</t>
+  </si>
+  <si>
+    <t>trottier.sebastien@cegepvicto.ca</t>
+  </si>
+  <si>
+    <t>https://teams.microsoft.com/l/chat/0/0?tenantId=9d6cf526-ad81-46f8-a73a-a507aaf06cda&amp;users=TROTTIER.SEBASTIEN@cegepvicto.ca</t>
   </si>
 </sst>
 </file>
@@ -583,7 +580,7 @@
         <v>13</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>14</v>
@@ -600,14 +597,13 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="2" t="s">
-        <v>35</v>
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="E3" t="s">
         <v>9</v>
@@ -616,18 +612,19 @@
         <v>10</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>32</v>
+        <v>20</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
         <v>9</v>
@@ -636,7 +633,7 @@
         <v>10</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -645,7 +642,7 @@
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="2" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>24</v>
@@ -662,14 +659,16 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="1"/>
+        <v>16</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>17</v>
+      </c>
       <c r="C6" s="2" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="E6" t="s">
         <v>9</v>
@@ -678,21 +677,19 @@
         <v>10</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>18</v>
+        <v>26</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>27</v>
       </c>
       <c r="E7" t="s">
         <v>9</v>
@@ -701,19 +698,19 @@
         <v>10</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="E8" t="s">
         <v>9</v>
@@ -722,30 +719,31 @@
         <v>10</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G7">
-    <sortCondition ref="A2:A7"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G6">
+    <sortCondition ref="A2:A6"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="D4" r:id="rId1" xr:uid="{F789545C-CEF6-4B3A-9358-1A6F9E968CF2}"/>
-    <hyperlink ref="G4" r:id="rId2" xr:uid="{142F557C-F7AB-411D-B17A-5FCFF3CE21F9}"/>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{F789545C-CEF6-4B3A-9358-1A6F9E968CF2}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{142F557C-F7AB-411D-B17A-5FCFF3CE21F9}"/>
     <hyperlink ref="D2" r:id="rId3" xr:uid="{47C36387-4B68-48E7-B056-2081D1996CF5}"/>
     <hyperlink ref="G2" r:id="rId4" xr:uid="{F550D781-4855-4E10-88FA-3A222809FFB7}"/>
-    <hyperlink ref="D7" r:id="rId5" xr:uid="{4C97C5B1-71FC-4BB8-8E2C-430E1A58D443}"/>
-    <hyperlink ref="G7" r:id="rId6" xr:uid="{F77BBB30-0E91-4834-992D-8C3E6F3FF743}"/>
-    <hyperlink ref="D3" r:id="rId7" xr:uid="{44F3169D-D34E-464F-A7BB-69732F62CD5B}"/>
-    <hyperlink ref="G3" r:id="rId8" xr:uid="{F739B185-8900-4D37-A986-42B107B5BD3B}"/>
-    <hyperlink ref="D5" r:id="rId9" xr:uid="{70C39852-F2CE-4E7F-AB0A-5CA460ECC68C}"/>
-    <hyperlink ref="G5" r:id="rId10" xr:uid="{263A76BA-B256-4A29-B498-E208EBF8E687}"/>
-    <hyperlink ref="D6" r:id="rId11" xr:uid="{8800F2D9-30C8-4D1C-9E71-40C42A1B9FC3}"/>
-    <hyperlink ref="G6" r:id="rId12" xr:uid="{90E6A9A5-6765-442D-8285-2B88419E6497}"/>
-    <hyperlink ref="D8" r:id="rId13" xr:uid="{2DFF4878-77A7-3147-BB6A-6F99564224C2}"/>
-    <hyperlink ref="G8" r:id="rId14" xr:uid="{0342F727-AE7C-6640-AFBE-6581114A221F}"/>
-    <hyperlink ref="C8" r:id="rId15" display="https://avatar.iran.liara.run/public/boy" xr:uid="{F3C9B75E-3DE9-B24C-AE26-1DB2B3BEBC66}"/>
+    <hyperlink ref="D6" r:id="rId5" xr:uid="{4C97C5B1-71FC-4BB8-8E2C-430E1A58D443}"/>
+    <hyperlink ref="G6" r:id="rId6" xr:uid="{F77BBB30-0E91-4834-992D-8C3E6F3FF743}"/>
+    <hyperlink ref="D4" r:id="rId7" xr:uid="{70C39852-F2CE-4E7F-AB0A-5CA460ECC68C}"/>
+    <hyperlink ref="G4" r:id="rId8" xr:uid="{263A76BA-B256-4A29-B498-E208EBF8E687}"/>
+    <hyperlink ref="D5" r:id="rId9" xr:uid="{8800F2D9-30C8-4D1C-9E71-40C42A1B9FC3}"/>
+    <hyperlink ref="G5" r:id="rId10" xr:uid="{90E6A9A5-6765-442D-8285-2B88419E6497}"/>
+    <hyperlink ref="D7" r:id="rId11" xr:uid="{2DFF4878-77A7-3147-BB6A-6F99564224C2}"/>
+    <hyperlink ref="G7" r:id="rId12" xr:uid="{0342F727-AE7C-6640-AFBE-6581114A221F}"/>
+    <hyperlink ref="C7" r:id="rId13" display="https://avatar.iran.liara.run/public/boy" xr:uid="{F3C9B75E-3DE9-B24C-AE26-1DB2B3BEBC66}"/>
+    <hyperlink ref="D8" r:id="rId14" display="tousignant.simon@cegepvicto.ca" xr:uid="{D6FF0BEA-A8BD-4E47-87EA-BC28501D9F3E}"/>
+    <hyperlink ref="G8" r:id="rId15" xr:uid="{8FBFFCC4-AE93-4C4F-8AB4-47F37BF23E43}"/>
+    <hyperlink ref="C8" r:id="rId16" display="https://avatar.iran.liara.run/public/boy" xr:uid="{746228E8-5E43-A646-970E-5C949E89D34E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>